<commit_message>
Added Testcases Execution of My Health benefits, Insurance KYC, Dream Gift and Query List module.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\04_Redemptions\Redemptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2576C3-641C-4F7F-AD2D-00AE36DA9AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F7D82E-5690-4E6D-9A0A-4389B46C1481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="112">
   <si>
     <t>INFLUENCER_ACCOUNT</t>
   </si>
@@ -1609,12 +1609,6 @@
     <t xml:space="preserve">
 summary_clickon_otpverfy_verifybtn
 verify_summary_mandatoryfields_error</t>
-  </si>
-  <si>
-    <t>summary_clickon_checkout
-summary_clickon_checkout
-summary_clickon_declaration_acceptbtn
-verify_summary_otpverfy_title</t>
   </si>
 </sst>
 </file>
@@ -2802,7 +2796,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -2816,7 +2810,7 @@
         <v>92</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="18"/>

</xml_diff>

<commit_message>
Mac- Resolved Failed Test Cases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\04_Redemptions\Redemptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53918775-7383-498A-887F-D814A0FFCC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A25DCF-D97D-4E06-92E7-3DB85C1F0502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="113">
   <si>
     <t>INFLUENCER_ACCOUNT</t>
   </si>
@@ -1609,6 +1609,12 @@
     <t xml:space="preserve">
 summary_clickon_otpverfy_verifybtn
 verify_summary_mandatoryfields_error</t>
+  </si>
+  <si>
+    <t>summary_clickon_checkout
+summary_clickon_checkout
+summary_clickon_declaration_acceptbtn
+verify_summary_otpverfy_title</t>
   </si>
 </sst>
 </file>
@@ -2761,7 +2767,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -2775,7 +2781,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>

</xml_diff>

<commit_message>
Resolved- MyWebSite Failed TestCases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\04_Redemptions\Redemptions\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A25DCF-D97D-4E06-92E7-3DB85C1F0502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="TestCases" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet r:id="rId1" sheetId="1" name="TestCases"/>
+    <sheet r:id="rId2" sheetId="2" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="112">
   <si>
     <t>INFLUENCER_ACCOUNT</t>
   </si>
@@ -1606,11 +1600,6 @@
 navigatebacktodashboardpage</t>
   </si>
   <si>
-    <t xml:space="preserve">
-summary_clickon_otpverfy_verifybtn
-verify_summary_mandatoryfields_error</t>
-  </si>
-  <si>
     <t>summary_clickon_checkout
 summary_clickon_checkout
 summary_clickon_declaration_acceptbtn
@@ -1620,8 +1609,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1632,48 +1622,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFffffff"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1686,17 +1642,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0070C0"/>
+        <fgColor rgb="FF0070c0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF96DCF8"/>
+        <fgColor rgb="FF96dcf8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFffffff"/>
       </patternFill>
     </fill>
   </fills>
@@ -1710,16 +1666,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </left>
       <right style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </right>
       <top style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1734,7 +1690,7 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1746,10 +1702,10 @@
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1779,96 +1735,104 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="30">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1879,10 +1843,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1920,71 +1884,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2012,7 +1976,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2035,11 +1999,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2048,13 +2012,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2064,7 +2028,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2073,7 +2037,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2082,7 +2046,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2090,10 +2054,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2158,32 +2122,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="74.1796875" style="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40.54296875" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="40.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" style="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.453125" style="26" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.26953125" style="26" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="24" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="24" width="28.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="25" width="74.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="24" width="47.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="26" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="27" width="6.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="26" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="27" width="19.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="27" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="28" width="8.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="29" width="32.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="29" width="30.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="24" width="11.719285714285713" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2236,7 +2201,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="246.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -2273,7 +2238,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -2283,10 +2248,10 @@
       <c r="C3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="11" t="s">
         <v>28</v>
       </c>
       <c r="F3" s="14"/>
@@ -2296,9 +2261,9 @@
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
       <c r="P3" s="9" t="s">
         <v>29</v>
       </c>
@@ -2306,7 +2271,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
@@ -2316,30 +2281,30 @@
       <c r="C4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="16" t="s">
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="18"/>
+      <c r="P4" s="16"/>
       <c r="Q4" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -2349,32 +2314,32 @@
       <c r="C5" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="16" t="s">
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="O5" s="17"/>
-      <c r="P5" s="19" t="s">
+      <c r="O5" s="15"/>
+      <c r="P5" s="17" t="s">
         <v>38</v>
       </c>
       <c r="Q5" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -2384,26 +2349,26 @@
       <c r="C6" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
       <c r="I6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="16" t="s">
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="O6" s="17"/>
+      <c r="O6" s="15"/>
       <c r="P6" s="9" t="s">
         <v>38</v>
       </c>
@@ -2411,7 +2376,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2421,24 +2386,24 @@
       <c r="C7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
       <c r="I7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
       <c r="P7" s="9" t="s">
         <v>48</v>
       </c>
@@ -2446,7 +2411,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -2456,24 +2421,24 @@
       <c r="C8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="11" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="16" t="s">
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="O8" s="17"/>
+      <c r="O8" s="15"/>
       <c r="P8" s="9" t="s">
         <v>38</v>
       </c>
@@ -2481,7 +2446,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
@@ -2491,24 +2456,24 @@
       <c r="C9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="16" t="s">
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="O9" s="17"/>
+      <c r="O9" s="15"/>
       <c r="P9" s="9" t="s">
         <v>38</v>
       </c>
@@ -2516,7 +2481,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -2526,24 +2491,24 @@
       <c r="C10" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="11" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="16" t="s">
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="O10" s="17"/>
+      <c r="O10" s="15"/>
       <c r="P10" s="9" t="s">
         <v>38</v>
       </c>
@@ -2551,7 +2516,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -2561,24 +2526,24 @@
       <c r="C11" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="11" t="s">
         <v>65</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="16" t="s">
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O11" s="17"/>
+      <c r="O11" s="15"/>
       <c r="P11" s="9" t="s">
         <v>38</v>
       </c>
@@ -2586,7 +2551,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -2596,26 +2561,26 @@
       <c r="C12" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
       <c r="L12" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="M12" s="17"/>
-      <c r="N12" s="16" t="s">
+      <c r="M12" s="15"/>
+      <c r="N12" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O12" s="17"/>
+      <c r="O12" s="15"/>
       <c r="P12" s="9" t="s">
         <v>38</v>
       </c>
@@ -2623,7 +2588,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -2633,22 +2598,22 @@
       <c r="C13" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
-      <c r="O13" s="17"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+      <c r="O13" s="15"/>
       <c r="P13" s="9" t="s">
         <v>74</v>
       </c>
@@ -2656,20 +2621,20 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="203" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
       <c r="A14" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="20" t="s">
+      <c r="B14" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="19" t="s">
         <v>77</v>
       </c>
       <c r="F14" s="12" t="s">
@@ -2678,30 +2643,30 @@
       <c r="G14" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="H14" s="20" t="s">
+      <c r="H14" s="18" t="s">
         <v>78</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="K14" s="20" t="s">
+      <c r="K14" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="L14" s="20" t="s">
+      <c r="L14" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="M14" s="22"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="22"/>
+      <c r="M14" s="20"/>
+      <c r="N14" s="20"/>
+      <c r="O14" s="20"/>
       <c r="P14" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="Q14" s="20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="Q14" s="18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
       <c r="A15" s="9" t="s">
         <v>17</v>
       </c>
@@ -2711,22 +2676,22 @@
       <c r="C15" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="11" t="s">
         <v>84</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
-      <c r="O15" s="17"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
       <c r="P15" s="9" t="s">
         <v>86</v>
       </c>
@@ -2734,7 +2699,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -2744,22 +2709,22 @@
       <c r="C16" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
       <c r="P16" s="9" t="s">
         <v>90</v>
       </c>
@@ -2767,7 +2732,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -2777,22 +2742,22 @@
       <c r="C17" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
+      <c r="E17" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
       <c r="P17" s="9" t="s">
         <v>94</v>
       </c>
@@ -2800,7 +2765,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -2810,23 +2775,24 @@
       <c r="C18" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="N18" s="16" t="s">
+      <c r="E18" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="O18" s="17"/>
+      <c r="O18" s="15"/>
       <c r="P18" s="9" t="s">
         <v>38</v>
       </c>
@@ -2834,7 +2800,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
       <c r="A19" s="9" t="s">
         <v>17</v>
       </c>
@@ -2844,24 +2810,24 @@
       <c r="C19" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="24" t="s">
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
       <c r="P19" s="9" t="s">
         <v>103</v>
       </c>
@@ -2869,7 +2835,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
       <c r="A20" s="9" t="s">
         <v>17</v>
       </c>
@@ -2879,22 +2845,22 @@
       <c r="C20" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="11" t="s">
         <v>105</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
       <c r="P20" s="9" t="s">
         <v>107</v>
       </c>
@@ -2902,7 +2868,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="60.75">
       <c r="A21" s="9" t="s">
         <v>17</v>
       </c>
@@ -2912,22 +2878,22 @@
       <c r="C21" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="E21" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
       <c r="P21" s="9" t="s">
         <v>90</v>
       </c>
@@ -2941,32 +2907,33 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:Q22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="74.1796875" style="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40.54296875" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="40.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" style="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.453125" style="26" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.26953125" style="26" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.81640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="24" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="24" width="28.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="25" width="74.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="24" width="47.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="26" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="27" width="6.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="26" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="27" width="19.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="27" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="28" width="8.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="29" width="32.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="29" width="30.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="24" width="11.719285714285713" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3019,7 +2986,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -3056,7 +3023,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -3066,10 +3033,10 @@
       <c r="C3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="11" t="s">
         <v>28</v>
       </c>
       <c r="F3" s="14"/>
@@ -3079,9 +3046,9 @@
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
       <c r="P3" s="9" t="s">
         <v>29</v>
       </c>
@@ -3089,7 +3056,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
@@ -3099,30 +3066,30 @@
       <c r="C4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="16" t="s">
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="18"/>
+      <c r="P4" s="16"/>
       <c r="Q4" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -3132,32 +3099,32 @@
       <c r="C5" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="16" t="s">
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="O5" s="17"/>
-      <c r="P5" s="19" t="s">
+      <c r="O5" s="15"/>
+      <c r="P5" s="17" t="s">
         <v>38</v>
       </c>
       <c r="Q5" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -3167,26 +3134,26 @@
       <c r="C6" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
       <c r="I6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="16" t="s">
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="O6" s="17"/>
+      <c r="O6" s="15"/>
       <c r="P6" s="9" t="s">
         <v>38</v>
       </c>
@@ -3194,7 +3161,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3204,24 +3171,24 @@
       <c r="C7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
       <c r="I7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
       <c r="P7" s="9" t="s">
         <v>48</v>
       </c>
@@ -3229,7 +3196,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -3239,24 +3206,24 @@
       <c r="C8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="11" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="16" t="s">
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="O8" s="17"/>
+      <c r="O8" s="15"/>
       <c r="P8" s="9" t="s">
         <v>38</v>
       </c>
@@ -3264,7 +3231,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
@@ -3274,24 +3241,24 @@
       <c r="C9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="16" t="s">
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="O9" s="17"/>
+      <c r="O9" s="15"/>
       <c r="P9" s="9" t="s">
         <v>38</v>
       </c>
@@ -3299,7 +3266,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -3309,24 +3276,24 @@
       <c r="C10" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="11" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="16" t="s">
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="O10" s="17"/>
+      <c r="O10" s="15"/>
       <c r="P10" s="9" t="s">
         <v>38</v>
       </c>
@@ -3334,7 +3301,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -3344,24 +3311,24 @@
       <c r="C11" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="16" t="s">
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="O11" s="17"/>
+      <c r="O11" s="15"/>
       <c r="P11" s="9" t="s">
         <v>38</v>
       </c>
@@ -3369,7 +3336,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -3379,24 +3346,24 @@
       <c r="C12" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="11" t="s">
         <v>65</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="16" t="s">
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O12" s="17"/>
+      <c r="O12" s="15"/>
       <c r="P12" s="9" t="s">
         <v>38</v>
       </c>
@@ -3404,7 +3371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -3414,26 +3381,26 @@
       <c r="C13" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
       <c r="L13" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="M13" s="17"/>
-      <c r="N13" s="16" t="s">
+      <c r="M13" s="15"/>
+      <c r="N13" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O13" s="17"/>
+      <c r="O13" s="15"/>
       <c r="P13" s="9" t="s">
         <v>38</v>
       </c>
@@ -3441,7 +3408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
@@ -3451,22 +3418,22 @@
       <c r="C14" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
       <c r="P14" s="9" t="s">
         <v>74</v>
       </c>
@@ -3474,20 +3441,20 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="20" t="s">
+      <c r="B15" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="D15" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="19" t="s">
         <v>77</v>
       </c>
       <c r="F15" s="12" t="s">
@@ -3496,30 +3463,30 @@
       <c r="G15" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="18" t="s">
         <v>78</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="K15" s="20" t="s">
+      <c r="K15" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="L15" s="20" t="s">
+      <c r="L15" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="20"/>
       <c r="P15" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="Q15" s="20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Q15" s="18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -3529,22 +3496,22 @@
       <c r="C16" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="11" t="s">
         <v>84</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
       <c r="P16" s="9" t="s">
         <v>86</v>
       </c>
@@ -3552,7 +3519,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -3562,22 +3529,22 @@
       <c r="C17" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
       <c r="P17" s="9" t="s">
         <v>90</v>
       </c>
@@ -3585,7 +3552,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -3595,22 +3562,22 @@
       <c r="C18" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
       <c r="P18" s="9" t="s">
         <v>94</v>
       </c>
@@ -3618,7 +3585,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="9" t="s">
         <v>17</v>
       </c>
@@ -3628,23 +3595,24 @@
       <c r="C19" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="N19" s="16" t="s">
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="O19" s="17"/>
+      <c r="O19" s="15"/>
       <c r="P19" s="9" t="s">
         <v>38</v>
       </c>
@@ -3652,7 +3620,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="9" t="s">
         <v>17</v>
       </c>
@@ -3662,24 +3630,24 @@
       <c r="C20" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="24" t="s">
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
       <c r="P20" s="9" t="s">
         <v>103</v>
       </c>
@@ -3687,7 +3655,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="9" t="s">
         <v>17</v>
       </c>
@@ -3697,22 +3665,22 @@
       <c r="C21" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="11" t="s">
         <v>105</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
       <c r="P21" s="9" t="s">
         <v>107</v>
       </c>
@@ -3720,7 +3688,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="9" t="s">
         <v>17</v>
       </c>
@@ -3730,22 +3698,22 @@
       <c r="C22" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
       <c r="P22" s="9" t="s">
         <v>90</v>
       </c>

</xml_diff>

<commit_message>
Resolved Failed test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/04_Redemptions/Redemptions/04_RedemptionSummaryPageTest.xlsx
@@ -1,21 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\04_Redemptions\Redemptions\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AED1653-B44B-498E-B4DD-23107B875310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="TestCases"/>
-    <sheet r:id="rId2" sheetId="2" name="Sheet1"/>
+    <sheet name="TestCases" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="113">
   <si>
     <t>INFLUENCER_ACCOUNT</t>
   </si>
@@ -1605,13 +1624,16 @@
 summary_clickon_declaration_acceptbtn
 verify_summary_otpverfy_title</t>
   </si>
+  <si>
+    <t xml:space="preserve">summary_clickon_cancelbtn
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1622,7 +1644,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFffffff"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
@@ -1630,6 +1652,34 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1642,17 +1692,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0070c0"/>
+        <fgColor rgb="FF0070C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF96dcf8"/>
+        <fgColor rgb="FF96DCF8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffffff"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -1666,16 +1716,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1690,7 +1740,7 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1702,10 +1752,10 @@
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1735,104 +1785,104 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+  <cellXfs count="29">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1843,10 +1893,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1884,71 +1934,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1976,7 +2026,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1999,11 +2049,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2012,13 +2062,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2028,7 +2078,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2037,7 +2087,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2046,7 +2096,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2054,10 +2104,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2122,33 +2172,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="24" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="24" width="28.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="25" width="74.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="24" width="47.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="26" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="27" width="6.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="26" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="27" width="19.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="27" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="28" width="8.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="29" width="32.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="29" width="30.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="24" width="11.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="20.90625" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.7265625" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="95.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.6328125" style="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" style="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.08984375" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.54296875" style="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.90625" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.54296875" style="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.54296875" style="26" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.36328125" style="26" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.81640625" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.90625" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.7265625" style="28" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="107.81640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.08984375" style="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row r="1" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2251,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row r="2" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -2238,7 +2288,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row r="3" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -2271,7 +2321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row r="4" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
@@ -2304,7 +2354,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row r="5" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -2339,7 +2389,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row r="6" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -2376,7 +2426,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row r="7" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2411,7 +2461,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row r="8" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -2446,7 +2496,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row r="9" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
@@ -2481,7 +2531,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row r="10" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -2516,7 +2566,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row r="11" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -2551,7 +2601,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row r="12" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -2588,7 +2638,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row r="13" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -2602,7 +2652,7 @@
         <v>72</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>73</v>
+        <v>112</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -2621,7 +2671,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row r="14" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>17</v>
       </c>
@@ -2666,7 +2716,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row r="15" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>17</v>
       </c>
@@ -2699,7 +2749,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row r="16" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -2732,7 +2782,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row r="17" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -2765,7 +2815,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row r="18" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -2788,7 +2838,6 @@
       <c r="J18" s="16"/>
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>
-      <c r="M18" s="21"/>
       <c r="N18" s="11" t="s">
         <v>98</v>
       </c>
@@ -2800,7 +2849,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row r="19" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>17</v>
       </c>
@@ -2835,7 +2884,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+    <row r="20" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>17</v>
       </c>
@@ -2868,7 +2917,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="60.75">
+    <row r="21" spans="1:17" ht="60.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>17</v>
       </c>
@@ -2907,33 +2956,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:Q22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="24" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="24" width="28.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="25" width="74.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="24" width="47.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="26" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="27" width="6.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="26" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="27" width="19.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="27" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="26" width="40.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="28" width="8.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="29" width="32.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="29" width="30.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="23" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="24" width="11.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="20.81640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.1796875" style="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" style="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.81640625" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.1796875" style="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.1796875" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="40.54296875" style="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="40.54296875" style="26" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.453125" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="30.26953125" style="28" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.81640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.7265625" style="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2986,7 +3034,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -3023,7 +3071,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -3056,7 +3104,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
@@ -3089,7 +3137,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -3124,7 +3172,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -3161,7 +3209,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3196,7 +3244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -3231,7 +3279,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
@@ -3266,7 +3314,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -3301,7 +3349,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -3336,7 +3384,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -3371,7 +3419,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -3408,7 +3456,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
@@ -3441,7 +3489,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>17</v>
       </c>
@@ -3486,7 +3534,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -3519,7 +3567,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -3552,7 +3600,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -3585,7 +3633,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>17</v>
       </c>
@@ -3608,7 +3656,6 @@
       <c r="J19" s="16"/>
       <c r="K19" s="16"/>
       <c r="L19" s="16"/>
-      <c r="M19" s="21"/>
       <c r="N19" s="11" t="s">
         <v>98</v>
       </c>
@@ -3620,7 +3667,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>17</v>
       </c>
@@ -3655,7 +3702,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>17</v>
       </c>
@@ -3688,7 +3735,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>17</v>
       </c>

</xml_diff>